<commit_message>
feat: reset cell merges in Code.gs and remove temporary Excel lock file
</commit_message>
<xml_diff>
--- a/KALKULATOR TAPLAK MEJA.xlsx
+++ b/KALKULATOR TAPLAK MEJA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afiffaizin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Development\AppScript-Calculator-Taplak\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C16B758-4959-4D3E-9F37-E75D6C76A282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6659E887-E419-492E-9E9A-604945474100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hasil" sheetId="1" r:id="rId1"/>
@@ -143,18 +143,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -383,30 +383,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="D1" s="1"/>
-      <c r="F1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="8"/>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
       <c r="D2" s="1"/>
-      <c r="F2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="6">
-        <v>7</v>
-      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
@@ -418,11 +406,11 @@
       <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="6">
-        <v>4</v>
+      <c r="F3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -435,8 +423,21 @@
       <c r="C4" s="4">
         <v>80</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2"/>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="F5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="6">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C2"/>
@@ -453,8 +454,8 @@
   <dimension ref="A3:L7"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A3" s="10" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="8"/>
@@ -462,7 +463,7 @@
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
       <c r="F3" s="2"/>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="10" t="s">
         <v>2</v>
       </c>
       <c r="I3" s="8"/>
@@ -470,27 +471,27 @@
       <c r="K3" s="8"/>
       <c r="L3" s="8"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+    <row r="4" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="7" t="s">
         <v>4</v>
       </c>
       <c r="E4" s="8"/>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="7" t="s">
         <v>3</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="7" t="s">
         <v>4</v>
       </c>
       <c r="L4" s="8"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>80</v>
       </c>
@@ -522,22 +523,22 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="10">
+    <row r="6" spans="1:12" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A6" s="9">
         <v>350</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <v>200</v>
       </c>
       <c r="E6" s="8"/>
-      <c r="H6" s="10">
+      <c r="H6" s="9">
         <v>200</v>
       </c>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
-      <c r="K6" s="10">
+      <c r="K6" s="9">
         <v>200</v>
       </c>
       <c r="L6" s="8"/>

</xml_diff>